<commit_message>
docs: deliver engineering artifact content and audience export contracts
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/engineering-artifacts-template.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/engineering-artifacts-template.xlsx
@@ -33,14 +33,16 @@
     <sheet name="23 Guidance and Handover" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="24 Vocabulary" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="25 Audience Profiles" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="26 Source Bindings" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="27 Source Manifest" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'00 Read Me'!$1:$4,'00 Read Me'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'00 Read Me'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'01 Control'!$1:$4,'01 Control'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Control'!$A$1:$C$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Control'!$A$1:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'02 Artifact Register'!$1:$4,'02 Artifact Register'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'02 Artifact Register'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'02 Artifact Register'!$A$1:$L$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'03 Sources'!$1:$4,'03 Sources'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'03 Sources'!$A$1:$G$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'04 Requirements'!$1:$4,'04 Requirements'!$A:$A</definedName>
@@ -84,9 +86,13 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="23">'23 Guidance and Handover'!$1:$4,'23 Guidance and Handover'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="23">'23 Guidance and Handover'!$A$1:$H$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="24">'24 Vocabulary'!$1:$4,'24 Vocabulary'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="24">'24 Vocabulary'!$A$1:$C$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="24">'24 Vocabulary'!$A$1:$C$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="25">'25 Audience Profiles'!$1:$4,'25 Audience Profiles'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="25">'25 Audience Profiles'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="26">'26 Source Bindings'!$1:$4,'26 Source Bindings'!$A:$A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="26">'26 Source Bindings'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="27">'27 Source Manifest'!$1:$4,'27 Source Manifest'!$A:$A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="27">'27 Source Manifest'!$A$1:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,8 +463,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EngineeringTemplate01" displayName="EngineeringTemplate01" ref="A4:C21" headerRowCount="1">
-  <autoFilter ref="A4:C21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EngineeringTemplate01" displayName="EngineeringTemplate01" ref="A4:C25" headerRowCount="1">
+  <autoFilter ref="A4:C25"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Value"/>
@@ -559,8 +565,8 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="EngineeringTemplate24" displayName="EngineeringTemplate24" ref="A4:C25" headerRowCount="1">
-  <autoFilter ref="A4:C25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="EngineeringTemplate24" displayName="EngineeringTemplate24" ref="A4:C31" headerRowCount="1">
+  <autoFilter ref="A4:C31"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Field"/>
     <tableColumn id="2" name="Value"/>
@@ -583,10 +589,47 @@
 </table>
 </file>
 
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="EngineeringTemplate26" displayName="EngineeringTemplate26" ref="A4:K5" headerRowCount="1">
+  <autoFilter ref="A4:K5"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="Binding ID"/>
+    <tableColumn id="2" name="Record Type"/>
+    <tableColumn id="3" name="Record ID"/>
+    <tableColumn id="4" name="Native Owner ID"/>
+    <tableColumn id="5" name="Source Path"/>
+    <tableColumn id="6" name="Source Kind"/>
+    <tableColumn id="7" name="Source Field"/>
+    <tableColumn id="8" name="Source Locator"/>
+    <tableColumn id="9" name="Source Text SHA-256"/>
+    <tableColumn id="10" name="Source File SHA-256"/>
+    <tableColumn id="11" name="Binding Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="EngineeringTemplate27" displayName="EngineeringTemplate27" ref="A4:H5" headerRowCount="1">
+  <autoFilter ref="A4:H5"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Source ID"/>
+    <tableColumn id="2" name="Source Kind"/>
+    <tableColumn id="3" name="Path"/>
+    <tableColumn id="4" name="Selector"/>
+    <tableColumn id="5" name="Revision"/>
+    <tableColumn id="6" name="SHA-256"/>
+    <tableColumn id="7" name="Authority"/>
+    <tableColumn id="8" name="Full-Source Link"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EngineeringTemplate02" displayName="EngineeringTemplate02" ref="A4:J5" headerRowCount="1">
-  <autoFilter ref="A4:J5"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EngineeringTemplate02" displayName="EngineeringTemplate02" ref="A4:L5" headerRowCount="1">
+  <autoFilter ref="A4:L5"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Artifact ID"/>
     <tableColumn id="2" name="Type"/>
     <tableColumn id="3" name="Title"/>
@@ -595,8 +638,10 @@
     <tableColumn id="6" name="Markdown Path"/>
     <tableColumn id="7" name="Source Section"/>
     <tableColumn id="8" name="Source Revision"/>
-    <tableColumn id="9" name="Supersedes ID"/>
-    <tableColumn id="10" name="Machine Source Link"/>
+    <tableColumn id="9" name="Source SHA-256"/>
+    <tableColumn id="10" name="Source Authority"/>
+    <tableColumn id="11" name="Supersedes ID"/>
+    <tableColumn id="12" name="Machine Source Link"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -2616,7 +2661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2693,210 +2738,266 @@
     <row r="6" ht="39" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Artifact baseline</t>
+          <t>Namespace</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr"/>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Reference the reviewed Markdown baseline.</t>
+          <t>Explicitly confirm identity scope; never infer from a repository name.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="39" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Document version</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
+          <t>Contract version</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Keep template, document and product versions distinct.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+          <t>Content and export contract used by this generic library.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="39" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Template version</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
+          <t>Profile version</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr"/>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Version of this generic template asset.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="39" customHeight="1">
+          <t>Version of the selected audience projection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Source Markdown paths</t>
+          <t>Source manifest</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr"/>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Full artifact paths; source sections listed in Artifact Register.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+          <t>List every source file, authority, revision and exact hash in Source Manifest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="39" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Source revision</t>
+          <t>Artifact baseline</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr"/>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Actual source revision used to export.</t>
+          <t>Reference the reviewed Markdown baseline.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="39" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Source SHA-256</t>
+          <t>Document version</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr"/>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Hash actual source content, not this template.</t>
+          <t>Keep template, document and product versions distinct.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Author / owner</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr"/>
+          <t>Template version</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Use confirmed ownership.</t>
+          <t>Version of this generic template asset.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="39" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Requested action</t>
+          <t>Source Markdown paths</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr"/>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Research, planning, drafting, review or another agreed action.</t>
+          <t>Full artifact paths; source sections listed in Artifact Register.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Export ID</t>
+          <t>Source revision</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr"/>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Assign when producing a derived view.</t>
+          <t>Actual source revision used to export.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="39" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Audience / profile</t>
+          <t>Source SHA-256</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr"/>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Select relevant views; record profile/version.</t>
+          <t>Hash actual source content, not this template.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Generated UTC</t>
+          <t>Author / owner</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr"/>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Actual generation timestamp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
+          <t>Use confirmed ownership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="39" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Omitted content</t>
+          <t>Requested action</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr"/>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Declare omitted detail and why.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="39" customHeight="1">
+          <t>Research, planning, drafting, review or another agreed action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Full-source links</t>
+          <t>Export ID</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr"/>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Provide links to complete canonical artifacts.</t>
+          <t>Assign when producing a derived view.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="39" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Relevant blockers / limits</t>
+          <t>Audience / profile</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr"/>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Retain material blockers even in brief summaries.</t>
+          <t>Select relevant views; record profile/version.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Feedback source export</t>
+          <t>Generated UTC</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr"/>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Identify the baseline/export reviewed.</t>
+          <t>Actual generation timestamp.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="39" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Feedback reconciliation status</t>
+          <t>Omitted content</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr"/>
       <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Declare omitted views/fields and why; preserve relevant blockers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="39" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Full-source links</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Provide links to complete canonical artifacts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="39" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Relevant blockers / limits</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Retain material blockers even in brief summaries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Feedback source export</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr"/>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Identify the baseline/export reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="39" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Feedback reconciliation status</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr"/>
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Proposed, reviewed or reconciled, with evidence.</t>
         </is>
@@ -3603,7 +3704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4018,6 +4119,108 @@
       <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Record replaces another while preserving history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Relation</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>depends_on</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Record needs another record or outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Relation</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>refers_to</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Record links contextual source content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="39" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Binding Status</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Mapping proposed for review; not export-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="39" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Binding Status</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Reviewed association at the declared source hashes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="39" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Binding Status</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>unresolved</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Ambiguous or stale source association; export blocker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="39" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Binding Status</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>retired</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Removed/replaced association retained in history.</t>
         </is>
       </c>
     </row>
@@ -4244,31 +4447,32 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="58" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>02 Artifact Register</t>
+          <t>26 Source Bindings</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -4277,7 +4481,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -4285,7 +4489,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Identify complete Markdown records and explicitly linked authoritative machine sources.</t>
+          <t>Persist reviewed individual requirement/criterion associations without changing legacy schemas. Indices and hashes locate entries; they are not identities. Source drift needs reconciliation.</t>
         </is>
       </c>
     </row>
@@ -4304,52 +4508,57 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Artifact ID</t>
+          <t>Binding ID</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Record Type</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Record ID</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Native Owner ID</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Source Path</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Markdown Path</t>
+          <t>Source Kind</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Source Section</t>
+          <t>Source Field</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Source Revision</t>
+          <t>Source Locator</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Supersedes ID</t>
+          <t>Source Text SHA-256</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Machine Source Link</t>
+          <t>Source File SHA-256</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Binding Status</t>
         </is>
       </c>
     </row>
@@ -4364,6 +4573,289 @@
       <c r="H5" s="6" t="inlineStr"/>
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="2"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Generic blank template | Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="58" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>27 Source Manifest</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Blank template</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="75" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Identify every source used by a real export, including the binding registry. Exact byte hashes detect changed working-tree content; unavailable freshness remains explicit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Return to Read Me</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Source ID</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Source Kind</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Selector</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Revision</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>SHA-256</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Authority</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Full-Source Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="6" t="inlineStr"/>
+      <c r="B5" s="6" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="2"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Generic blank template | Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="58" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>02 Artifact Register</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Blank template</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Identify complete Markdown records and explicitly linked authoritative machine sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Return to Read Me</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Artifact ID</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Markdown Path</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Source Section</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Source Revision</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Source SHA-256</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Source Authority</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Supersedes ID</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Machine Source Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="6" t="inlineStr"/>
+      <c r="B5" s="6" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>